<commit_message>
Update notes for FM, GFM, and Time Series moving average
</commit_message>
<xml_diff>
--- a/Time Series/moving_average.xlsx
+++ b/Time Series/moving_average.xlsx
@@ -5,18 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hp\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MSQF\Semester III\Time Series\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54D264F3-3B20-4958-A9B4-22686398EAB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98AF9627-FACE-4471-957B-5D53B7D27CDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Moving Average" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
     <sheet name="03-09" sheetId="3" r:id="rId3"/>
     <sheet name="04-09" sheetId="4" r:id="rId4"/>
+    <sheet name="07-09" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="52">
   <si>
     <t>Year</t>
   </si>
@@ -181,6 +182,15 @@
   </si>
   <si>
     <t>SUM</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Smoothed (alpha = 0.8)</t>
+  </si>
+  <si>
+    <t>Trend (beta = 0.4)</t>
   </si>
 </sst>
 </file>
@@ -3187,15 +3197,15 @@
         <v>6.5</v>
       </c>
       <c r="C24" s="21">
-        <f>SUM(B21:B24)/4</f>
+        <f t="shared" ref="C24:C36" si="2">SUM(B21:B24)/4</f>
         <v>5.35</v>
       </c>
       <c r="D24" s="21">
-        <f t="shared" ref="D24:D34" si="2">SUM(C25:C26)/2</f>
+        <f t="shared" ref="D24:D34" si="3">SUM(C25:C26)/2</f>
         <v>5.7375000000000007</v>
       </c>
       <c r="E24" s="23">
-        <f t="shared" ref="E24:E34" si="3">B24/D24*100</f>
+        <f t="shared" ref="E24:E34" si="4">B24/D24*100</f>
         <v>113.28976034858387</v>
       </c>
       <c r="F24" s="20"/>
@@ -3210,15 +3220,15 @@
         <v>5.8</v>
       </c>
       <c r="C25" s="21">
-        <f>SUM(B22:B25)/4</f>
+        <f t="shared" si="2"/>
         <v>5.6000000000000005</v>
       </c>
       <c r="D25" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5.9749999999999996</v>
       </c>
       <c r="E25" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>97.071129707112974</v>
       </c>
       <c r="G25" s="24" t="s">
@@ -3237,15 +3247,15 @@
         <v>5.2</v>
       </c>
       <c r="C26" s="21">
-        <f>SUM(B23:B26)/4</f>
+        <f t="shared" si="2"/>
         <v>5.875</v>
       </c>
       <c r="D26" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6.1875</v>
       </c>
       <c r="E26" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>84.040404040404042</v>
       </c>
       <c r="F26" s="20"/>
@@ -3265,15 +3275,15 @@
         <v>6.8</v>
       </c>
       <c r="C27" s="21">
-        <f>SUM(B24:B27)/4</f>
+        <f t="shared" si="2"/>
         <v>6.0750000000000002</v>
       </c>
       <c r="D27" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6.3250000000000002</v>
       </c>
       <c r="E27" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>107.50988142292491</v>
       </c>
       <c r="F27" s="20"/>
@@ -3293,15 +3303,15 @@
         <v>7.4</v>
       </c>
       <c r="C28" s="21">
-        <f>SUM(B25:B28)/4</f>
+        <f t="shared" si="2"/>
         <v>6.3000000000000007</v>
       </c>
       <c r="D28" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6.3999999999999995</v>
       </c>
       <c r="E28" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>115.62500000000003</v>
       </c>
       <c r="F28" s="20"/>
@@ -3321,15 +3331,15 @@
         <v>6</v>
       </c>
       <c r="C29" s="21">
-        <f>SUM(B26:B29)/4</f>
+        <f t="shared" si="2"/>
         <v>6.35</v>
       </c>
       <c r="D29" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6.5374999999999996</v>
       </c>
       <c r="E29" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>91.778202676864254</v>
       </c>
       <c r="F29" s="20"/>
@@ -3349,15 +3359,15 @@
         <v>5.6</v>
       </c>
       <c r="C30" s="21">
-        <f>SUM(B27:B30)/4</f>
+        <f t="shared" si="2"/>
         <v>6.4499999999999993</v>
       </c>
       <c r="D30" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6.6750000000000007</v>
       </c>
       <c r="E30" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>83.8951310861423</v>
       </c>
       <c r="F30" s="20"/>
@@ -3372,15 +3382,15 @@
         <v>7.5</v>
       </c>
       <c r="C31" s="21">
-        <f>SUM(B28:B31)/4</f>
+        <f t="shared" si="2"/>
         <v>6.625</v>
       </c>
       <c r="D31" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6.7625000000000002</v>
       </c>
       <c r="E31" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>110.90573012939002</v>
       </c>
       <c r="F31" s="20"/>
@@ -3395,15 +3405,15 @@
         <v>7.8</v>
       </c>
       <c r="C32" s="21">
-        <f>SUM(B29:B32)/4</f>
+        <f t="shared" si="2"/>
         <v>6.7250000000000005</v>
       </c>
       <c r="D32" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6.8375000000000004</v>
       </c>
       <c r="E32" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>114.07678244972577</v>
       </c>
       <c r="F32" s="20"/>
@@ -3418,15 +3428,15 @@
         <v>6.3</v>
       </c>
       <c r="C33" s="21">
-        <f>SUM(B30:B33)/4</f>
+        <f t="shared" si="2"/>
         <v>6.8</v>
       </c>
       <c r="D33" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6.9375</v>
       </c>
       <c r="E33" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>90.810810810810807</v>
       </c>
       <c r="F33" s="20"/>
@@ -3441,15 +3451,15 @@
         <v>5.9</v>
       </c>
       <c r="C34" s="21">
-        <f>SUM(B31:B34)/4</f>
+        <f t="shared" si="2"/>
         <v>6.875</v>
       </c>
       <c r="D34" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>7.0750000000000002</v>
       </c>
       <c r="E34" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>83.392226148409904</v>
       </c>
       <c r="F34" s="20"/>
@@ -3464,7 +3474,7 @@
         <v>8</v>
       </c>
       <c r="C35" s="21">
-        <f>SUM(B32:B35)/4</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="D35" s="21"/>
@@ -3481,7 +3491,7 @@
         <v>8.4</v>
       </c>
       <c r="C36" s="21">
-        <f>SUM(B33:B36)/4</f>
+        <f t="shared" si="2"/>
         <v>7.15</v>
       </c>
       <c r="D36" s="21"/>
@@ -3495,4 +3505,267 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D973F176-01BA-48F1-B2A8-F5B7D16EF4F0}">
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="4" max="4" width="20.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.25" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" t="s">
+        <v>49</v>
+      </c>
+      <c r="J1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L1" t="s">
+        <v>50</v>
+      </c>
+      <c r="M1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>2010</v>
+      </c>
+      <c r="C2">
+        <v>1451</v>
+      </c>
+      <c r="D2">
+        <f>C2</f>
+        <v>1451</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>2010</v>
+      </c>
+      <c r="K2">
+        <v>1451</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2011</v>
+      </c>
+      <c r="C3">
+        <v>1499</v>
+      </c>
+      <c r="D3">
+        <f>0.8*C3+(1-0.8)*(C2*E2)</f>
+        <v>1199.2</v>
+      </c>
+      <c r="E3">
+        <f>0.4*(D3-D2)+(1-0.4)*E2</f>
+        <v>-100.71999999999998</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>2011</v>
+      </c>
+      <c r="K3">
+        <v>1499</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>2012</v>
+      </c>
+      <c r="C4">
+        <v>1686</v>
+      </c>
+      <c r="I4">
+        <v>3</v>
+      </c>
+      <c r="J4">
+        <v>2012</v>
+      </c>
+      <c r="K4">
+        <v>1686</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>2013</v>
+      </c>
+      <c r="C5">
+        <v>1764</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
+      </c>
+      <c r="J5">
+        <v>2013</v>
+      </c>
+      <c r="K5">
+        <v>1764</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>2014</v>
+      </c>
+      <c r="C6">
+        <v>1879</v>
+      </c>
+      <c r="I6">
+        <v>5</v>
+      </c>
+      <c r="J6">
+        <v>2014</v>
+      </c>
+      <c r="K6">
+        <v>1879</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>2015</v>
+      </c>
+      <c r="C7">
+        <v>1948</v>
+      </c>
+      <c r="I7">
+        <v>6</v>
+      </c>
+      <c r="J7">
+        <v>2015</v>
+      </c>
+      <c r="K7">
+        <v>1948</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>2016</v>
+      </c>
+      <c r="C8">
+        <v>2013</v>
+      </c>
+      <c r="I8">
+        <v>7</v>
+      </c>
+      <c r="J8">
+        <v>2016</v>
+      </c>
+      <c r="K8">
+        <v>2013</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>2017</v>
+      </c>
+      <c r="C9">
+        <v>2090</v>
+      </c>
+      <c r="I9">
+        <v>8</v>
+      </c>
+      <c r="J9">
+        <v>2017</v>
+      </c>
+      <c r="K9">
+        <v>2090</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>2018</v>
+      </c>
+      <c r="C10">
+        <v>2173</v>
+      </c>
+      <c r="I10">
+        <v>9</v>
+      </c>
+      <c r="J10">
+        <v>2018</v>
+      </c>
+      <c r="K10">
+        <v>2173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>2019</v>
+      </c>
+      <c r="C11">
+        <v>2286</v>
+      </c>
+      <c r="I11">
+        <v>10</v>
+      </c>
+      <c r="J11">
+        <v>2019</v>
+      </c>
+      <c r="K11">
+        <v>2286</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update notes: 08-09-2026 14:35
</commit_message>
<xml_diff>
--- a/Time Series/moving_average.xlsx
+++ b/Time Series/moving_average.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MSQF\Semester III\Time Series\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98AF9627-FACE-4471-957B-5D53B7D27CDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49C4E6BD-F7BA-4AB1-9540-8C71E16A1116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,6 +18,7 @@
     <sheet name="03-09" sheetId="3" r:id="rId3"/>
     <sheet name="04-09" sheetId="4" r:id="rId4"/>
     <sheet name="07-09" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet2" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="56">
   <si>
     <t>Year</t>
   </si>
@@ -191,13 +192,25 @@
   </si>
   <si>
     <t>Trend (beta = 0.4)</t>
+  </si>
+  <si>
+    <t>Row</t>
+  </si>
+  <si>
+    <t>Smoothed / Level</t>
+  </si>
+  <si>
+    <t>Trend</t>
+  </si>
+  <si>
+    <t>Forecast</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -216,6 +229,10 @@
     <font>
       <sz val="8"/>
       <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="3">
@@ -314,7 +331,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -381,6 +398,12 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -3509,7 +3532,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D973F176-01BA-48F1-B2A8-F5B7D16EF4F0}">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="4" max="4" width="20.25" bestFit="1" customWidth="1"/>
@@ -3765,7 +3788,273 @@
         <v>2286</v>
       </c>
     </row>
+    <row r="14" spans="1:13">
+      <c r="A14" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="C14" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" s="26" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
+      <c r="A15" s="20">
+        <v>1</v>
+      </c>
+      <c r="B15" s="20">
+        <v>2010</v>
+      </c>
+      <c r="C15" s="20">
+        <v>1451</v>
+      </c>
+      <c r="D15" s="27">
+        <f>C15</f>
+        <v>1451</v>
+      </c>
+      <c r="E15" s="27">
+        <f>C16-C15</f>
+        <v>48</v>
+      </c>
+      <c r="F15" s="27">
+        <f>D15+E15</f>
+        <v>1499</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
+      <c r="A16" s="20">
+        <v>2</v>
+      </c>
+      <c r="B16" s="20">
+        <v>2011</v>
+      </c>
+      <c r="C16" s="20">
+        <v>1499</v>
+      </c>
+      <c r="D16" s="27">
+        <f>0.8*C16+0.2*(D15+E15)</f>
+        <v>1499</v>
+      </c>
+      <c r="E16" s="27">
+        <f>0.4*(D16-D15)+0.6*E15</f>
+        <v>48</v>
+      </c>
+      <c r="F16" s="27">
+        <f>D16+E16</f>
+        <v>1547</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="20">
+        <v>3</v>
+      </c>
+      <c r="B17" s="20">
+        <v>2012</v>
+      </c>
+      <c r="C17" s="20">
+        <v>1686</v>
+      </c>
+      <c r="D17" s="27">
+        <f>0.8*C17+0.2*(D16+E16)</f>
+        <v>1658.2000000000003</v>
+      </c>
+      <c r="E17" s="27">
+        <f>0.4*(D17-D16)+0.6*E16</f>
+        <v>92.480000000000103</v>
+      </c>
+      <c r="F17" s="27">
+        <f>D17+E17</f>
+        <v>1750.6800000000003</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="20">
+        <v>4</v>
+      </c>
+      <c r="B18" s="20">
+        <v>2013</v>
+      </c>
+      <c r="C18" s="20">
+        <v>1764</v>
+      </c>
+      <c r="D18" s="27">
+        <f>0.8*C18+0.2*(D17+E17)</f>
+        <v>1761.3360000000002</v>
+      </c>
+      <c r="E18" s="27">
+        <f>0.4*(D18-D17)+0.6*E17</f>
+        <v>96.74240000000006</v>
+      </c>
+      <c r="F18" s="27">
+        <f>D18+E18</f>
+        <v>1858.0784000000003</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="20">
+        <v>5</v>
+      </c>
+      <c r="B19" s="20">
+        <v>2014</v>
+      </c>
+      <c r="C19" s="20">
+        <v>1879</v>
+      </c>
+      <c r="D19" s="27">
+        <f>0.8*C19+0.2*(D18+E18)</f>
+        <v>1874.8156800000002</v>
+      </c>
+      <c r="E19" s="27">
+        <f>0.4*(D19-D18)+0.6*E18</f>
+        <v>103.43731200000001</v>
+      </c>
+      <c r="F19" s="27">
+        <f>D19+E19</f>
+        <v>1978.2529920000002</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="20">
+        <v>6</v>
+      </c>
+      <c r="B20" s="20">
+        <v>2015</v>
+      </c>
+      <c r="C20" s="20">
+        <v>1948</v>
+      </c>
+      <c r="D20" s="27">
+        <f>0.8*C20+0.2*(D19+E19)</f>
+        <v>1954.0505984000001</v>
+      </c>
+      <c r="E20" s="27">
+        <f>0.4*(D20-D19)+0.6*E19</f>
+        <v>93.756354559999991</v>
+      </c>
+      <c r="F20" s="27">
+        <f>D20+E20</f>
+        <v>2047.8069529600002</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="20">
+        <v>7</v>
+      </c>
+      <c r="B21" s="20">
+        <v>2016</v>
+      </c>
+      <c r="C21" s="20">
+        <v>2013</v>
+      </c>
+      <c r="D21" s="27">
+        <f>0.8*C21+0.2*(D20+E20)</f>
+        <v>2019.961390592</v>
+      </c>
+      <c r="E21" s="27">
+        <f>0.4*(D21-D20)+0.6*E20</f>
+        <v>82.618129612799962</v>
+      </c>
+      <c r="F21" s="27">
+        <f>D21+E21</f>
+        <v>2102.5795202047998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="20">
+        <v>8</v>
+      </c>
+      <c r="B22" s="20">
+        <v>2017</v>
+      </c>
+      <c r="C22" s="20">
+        <v>2090</v>
+      </c>
+      <c r="D22" s="27">
+        <f>0.8*C22+0.2*(D21+E21)</f>
+        <v>2092.5159040409599</v>
+      </c>
+      <c r="E22" s="27">
+        <f>0.4*(D22-D21)+0.6*E21</f>
+        <v>78.592683147263898</v>
+      </c>
+      <c r="F22" s="27">
+        <f>D22+E22</f>
+        <v>2171.1085871882237</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="20">
+        <v>9</v>
+      </c>
+      <c r="B23" s="20">
+        <v>2018</v>
+      </c>
+      <c r="C23" s="20">
+        <v>2173</v>
+      </c>
+      <c r="D23" s="27">
+        <f>0.8*C23+0.2*(D22+E22)</f>
+        <v>2172.6217174376447</v>
+      </c>
+      <c r="E23" s="27">
+        <f>0.4*(D23-D22)+0.6*E22</f>
+        <v>79.197935247032291</v>
+      </c>
+      <c r="F23" s="27">
+        <f>D23+E23</f>
+        <v>2251.8196526846768</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="20">
+        <v>10</v>
+      </c>
+      <c r="B24" s="20">
+        <v>2019</v>
+      </c>
+      <c r="C24" s="20">
+        <v>2286</v>
+      </c>
+      <c r="D24" s="27">
+        <f>0.8*C24+0.2*(D23+E23)</f>
+        <v>2279.1639305369354</v>
+      </c>
+      <c r="E24" s="27">
+        <f>0.4*(D24-D23)+0.6*E23</f>
+        <v>90.135646387935623</v>
+      </c>
+      <c r="F24" s="27">
+        <f>D24+E24</f>
+        <v>2369.299576924871</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73D24AC6-6CB4-4F9B-9462-B818885DA0E0}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="4.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.75" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update notes: 09-09-2026 14:35
</commit_message>
<xml_diff>
--- a/Time Series/moving_average.xlsx
+++ b/Time Series/moving_average.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MSQF\Semester III\Time Series\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49C4E6BD-F7BA-4AB1-9540-8C71E16A1116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8BECB8D-BC4B-48E4-A6EE-7AA0953E898E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Moving Average" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="03-09" sheetId="3" r:id="rId3"/>
     <sheet name="04-09" sheetId="4" r:id="rId4"/>
     <sheet name="07-09" sheetId="5" r:id="rId5"/>
-    <sheet name="Sheet2" sheetId="6" r:id="rId6"/>
+    <sheet name="09-09" sheetId="7" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="56">
   <si>
     <t>Year</t>
   </si>
@@ -197,13 +197,13 @@
     <t>Row</t>
   </si>
   <si>
-    <t>Smoothed / Level</t>
-  </si>
-  <si>
-    <t>Trend</t>
-  </si>
-  <si>
     <t>Forecast</t>
+  </si>
+  <si>
+    <t>Trend (beta = 0.5)</t>
+  </si>
+  <si>
+    <t>Smoothed (alpha = 0.5)</t>
   </si>
 </sst>
 </file>
@@ -400,7 +400,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -3798,14 +3798,14 @@
       <c r="C14" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="D14" s="26" t="s">
+      <c r="D14" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" t="s">
+        <v>51</v>
+      </c>
+      <c r="F14" s="26" t="s">
         <v>53</v>
-      </c>
-      <c r="E14" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="F14" s="26" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -3827,7 +3827,7 @@
         <v>48</v>
       </c>
       <c r="F15" s="27">
-        <f>D15+E15</f>
+        <f t="shared" ref="F15:F24" si="0">D15+E15</f>
         <v>1499</v>
       </c>
     </row>
@@ -3842,15 +3842,15 @@
         <v>1499</v>
       </c>
       <c r="D16" s="27">
-        <f>0.8*C16+0.2*(D15+E15)</f>
+        <f t="shared" ref="D16:D24" si="1">0.8*C16+0.2*(D15+E15)</f>
         <v>1499</v>
       </c>
       <c r="E16" s="27">
-        <f>0.4*(D16-D15)+0.6*E15</f>
+        <f t="shared" ref="E16:E24" si="2">0.4*(D16-D15)+0.6*E15</f>
         <v>48</v>
       </c>
       <c r="F16" s="27">
-        <f>D16+E16</f>
+        <f t="shared" si="0"/>
         <v>1547</v>
       </c>
     </row>
@@ -3865,15 +3865,15 @@
         <v>1686</v>
       </c>
       <c r="D17" s="27">
-        <f>0.8*C17+0.2*(D16+E16)</f>
+        <f t="shared" si="1"/>
         <v>1658.2000000000003</v>
       </c>
       <c r="E17" s="27">
-        <f>0.4*(D17-D16)+0.6*E16</f>
+        <f t="shared" si="2"/>
         <v>92.480000000000103</v>
       </c>
       <c r="F17" s="27">
-        <f>D17+E17</f>
+        <f t="shared" si="0"/>
         <v>1750.6800000000003</v>
       </c>
     </row>
@@ -3888,15 +3888,15 @@
         <v>1764</v>
       </c>
       <c r="D18" s="27">
-        <f>0.8*C18+0.2*(D17+E17)</f>
+        <f t="shared" si="1"/>
         <v>1761.3360000000002</v>
       </c>
       <c r="E18" s="27">
-        <f>0.4*(D18-D17)+0.6*E17</f>
+        <f t="shared" si="2"/>
         <v>96.74240000000006</v>
       </c>
       <c r="F18" s="27">
-        <f>D18+E18</f>
+        <f t="shared" si="0"/>
         <v>1858.0784000000003</v>
       </c>
     </row>
@@ -3911,15 +3911,15 @@
         <v>1879</v>
       </c>
       <c r="D19" s="27">
-        <f>0.8*C19+0.2*(D18+E18)</f>
+        <f t="shared" si="1"/>
         <v>1874.8156800000002</v>
       </c>
       <c r="E19" s="27">
-        <f>0.4*(D19-D18)+0.6*E18</f>
+        <f t="shared" si="2"/>
         <v>103.43731200000001</v>
       </c>
       <c r="F19" s="27">
-        <f>D19+E19</f>
+        <f t="shared" si="0"/>
         <v>1978.2529920000002</v>
       </c>
     </row>
@@ -3934,15 +3934,15 @@
         <v>1948</v>
       </c>
       <c r="D20" s="27">
-        <f>0.8*C20+0.2*(D19+E19)</f>
+        <f t="shared" si="1"/>
         <v>1954.0505984000001</v>
       </c>
       <c r="E20" s="27">
-        <f>0.4*(D20-D19)+0.6*E19</f>
+        <f t="shared" si="2"/>
         <v>93.756354559999991</v>
       </c>
       <c r="F20" s="27">
-        <f>D20+E20</f>
+        <f t="shared" si="0"/>
         <v>2047.8069529600002</v>
       </c>
     </row>
@@ -3957,15 +3957,15 @@
         <v>2013</v>
       </c>
       <c r="D21" s="27">
-        <f>0.8*C21+0.2*(D20+E20)</f>
+        <f t="shared" si="1"/>
         <v>2019.961390592</v>
       </c>
       <c r="E21" s="27">
-        <f>0.4*(D21-D20)+0.6*E20</f>
+        <f t="shared" si="2"/>
         <v>82.618129612799962</v>
       </c>
       <c r="F21" s="27">
-        <f>D21+E21</f>
+        <f t="shared" si="0"/>
         <v>2102.5795202047998</v>
       </c>
     </row>
@@ -3980,15 +3980,15 @@
         <v>2090</v>
       </c>
       <c r="D22" s="27">
-        <f>0.8*C22+0.2*(D21+E21)</f>
+        <f t="shared" si="1"/>
         <v>2092.5159040409599</v>
       </c>
       <c r="E22" s="27">
-        <f>0.4*(D22-D21)+0.6*E21</f>
+        <f t="shared" si="2"/>
         <v>78.592683147263898</v>
       </c>
       <c r="F22" s="27">
-        <f>D22+E22</f>
+        <f t="shared" si="0"/>
         <v>2171.1085871882237</v>
       </c>
     </row>
@@ -4003,15 +4003,15 @@
         <v>2173</v>
       </c>
       <c r="D23" s="27">
-        <f>0.8*C23+0.2*(D22+E22)</f>
+        <f t="shared" si="1"/>
         <v>2172.6217174376447</v>
       </c>
       <c r="E23" s="27">
-        <f>0.4*(D23-D22)+0.6*E22</f>
+        <f t="shared" si="2"/>
         <v>79.197935247032291</v>
       </c>
       <c r="F23" s="27">
-        <f>D23+E23</f>
+        <f t="shared" si="0"/>
         <v>2251.8196526846768</v>
       </c>
     </row>
@@ -4026,15 +4026,15 @@
         <v>2286</v>
       </c>
       <c r="D24" s="27">
-        <f>0.8*C24+0.2*(D23+E23)</f>
+        <f t="shared" si="1"/>
         <v>2279.1639305369354</v>
       </c>
       <c r="E24" s="27">
-        <f>0.4*(D24-D23)+0.6*E23</f>
+        <f t="shared" si="2"/>
         <v>90.135646387935623</v>
       </c>
       <c r="F24" s="27">
-        <f>D24+E24</f>
+        <f t="shared" si="0"/>
         <v>2369.299576924871</v>
       </c>
     </row>
@@ -4044,17 +4044,281 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73D24AC6-6CB4-4F9B-9462-B818885DA0E0}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8CB44E7-2BB4-47B2-BF22-9D33AD8358A8}">
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="4.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.125" bestFit="1" customWidth="1"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="26" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="20">
+        <v>1</v>
+      </c>
+      <c r="B2" s="20">
+        <v>2010</v>
+      </c>
+      <c r="C2" s="20">
+        <v>1451</v>
+      </c>
+      <c r="D2" s="27">
+        <f>C2</f>
+        <v>1451</v>
+      </c>
+      <c r="E2" s="27">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <f>0</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="20">
+        <v>2</v>
+      </c>
+      <c r="B3" s="20">
+        <v>2011</v>
+      </c>
+      <c r="C3" s="20">
+        <v>1499</v>
+      </c>
+      <c r="D3" s="27">
+        <f>0.5*C3+(1-0.5)*(D2+E2)</f>
+        <v>1475</v>
+      </c>
+      <c r="E3" s="27">
+        <f>0.5*(D3-D2)+(1-0.5)*E2</f>
+        <v>12</v>
+      </c>
+      <c r="F3" s="27">
+        <f>D2+E2</f>
+        <v>1451</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="20">
+        <v>3</v>
+      </c>
+      <c r="B4" s="20">
+        <v>2012</v>
+      </c>
+      <c r="C4" s="20">
+        <v>1686</v>
+      </c>
+      <c r="D4" s="27">
+        <f t="shared" ref="D4:D11" si="0">0.5*C4+(1-0.5)*(D3+E3)</f>
+        <v>1586.5</v>
+      </c>
+      <c r="E4" s="27">
+        <f t="shared" ref="E4:E11" si="1">0.5*(D4-D3)+(1-0.5)*E3</f>
+        <v>61.75</v>
+      </c>
+      <c r="F4" s="27">
+        <f>D3+E3</f>
+        <v>1487</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="20">
+        <v>4</v>
+      </c>
+      <c r="B5" s="20">
+        <v>2013</v>
+      </c>
+      <c r="C5" s="20">
+        <v>1764</v>
+      </c>
+      <c r="D5" s="27">
+        <f t="shared" si="0"/>
+        <v>1706.125</v>
+      </c>
+      <c r="E5" s="27">
+        <f t="shared" si="1"/>
+        <v>90.6875</v>
+      </c>
+      <c r="F5" s="27">
+        <f>D4+E4</f>
+        <v>1648.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="20">
+        <v>5</v>
+      </c>
+      <c r="B6" s="20">
+        <v>2014</v>
+      </c>
+      <c r="C6" s="20">
+        <v>1879</v>
+      </c>
+      <c r="D6" s="27">
+        <f t="shared" si="0"/>
+        <v>1837.90625</v>
+      </c>
+      <c r="E6" s="27">
+        <f t="shared" si="1"/>
+        <v>111.234375</v>
+      </c>
+      <c r="F6" s="27">
+        <f>D5+E5</f>
+        <v>1796.8125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="20">
+        <v>6</v>
+      </c>
+      <c r="B7" s="20">
+        <v>2015</v>
+      </c>
+      <c r="C7" s="20">
+        <v>1948</v>
+      </c>
+      <c r="D7" s="27">
+        <f t="shared" si="0"/>
+        <v>1948.5703125</v>
+      </c>
+      <c r="E7" s="27">
+        <f t="shared" si="1"/>
+        <v>110.94921875</v>
+      </c>
+      <c r="F7" s="27">
+        <f>D6+E6</f>
+        <v>1949.140625</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="20">
+        <v>7</v>
+      </c>
+      <c r="B8" s="20">
+        <v>2016</v>
+      </c>
+      <c r="C8" s="20">
+        <v>2013</v>
+      </c>
+      <c r="D8" s="27">
+        <f t="shared" si="0"/>
+        <v>2036.259765625</v>
+      </c>
+      <c r="E8" s="27">
+        <f t="shared" si="1"/>
+        <v>99.3193359375</v>
+      </c>
+      <c r="F8" s="27">
+        <f>D7+E7</f>
+        <v>2059.51953125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="20">
+        <v>8</v>
+      </c>
+      <c r="B9" s="20">
+        <v>2017</v>
+      </c>
+      <c r="C9" s="20">
+        <v>2090</v>
+      </c>
+      <c r="D9" s="27">
+        <f t="shared" si="0"/>
+        <v>2112.78955078125</v>
+      </c>
+      <c r="E9" s="27">
+        <f t="shared" si="1"/>
+        <v>87.924560546875</v>
+      </c>
+      <c r="F9" s="27">
+        <f>D8+E8</f>
+        <v>2135.5791015625</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="20">
+        <v>9</v>
+      </c>
+      <c r="B10" s="20">
+        <v>2018</v>
+      </c>
+      <c r="C10" s="20">
+        <v>2173</v>
+      </c>
+      <c r="D10" s="27">
+        <f t="shared" si="0"/>
+        <v>2186.8570556640625</v>
+      </c>
+      <c r="E10" s="27">
+        <f t="shared" si="1"/>
+        <v>80.99603271484375</v>
+      </c>
+      <c r="F10" s="27">
+        <f>D9+E9</f>
+        <v>2200.714111328125</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="20">
+        <v>10</v>
+      </c>
+      <c r="B11" s="20">
+        <v>2019</v>
+      </c>
+      <c r="C11" s="20">
+        <v>2286</v>
+      </c>
+      <c r="D11" s="27">
+        <f t="shared" si="0"/>
+        <v>2276.9265441894531</v>
+      </c>
+      <c r="E11" s="27">
+        <f t="shared" si="1"/>
+        <v>85.532760620117188</v>
+      </c>
+      <c r="F11" s="27">
+        <f>D10+E10</f>
+        <v>2267.8530883789063</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="20">
+        <v>11</v>
+      </c>
+      <c r="B12" s="20">
+        <v>2020</v>
+      </c>
+      <c r="F12" s="27">
+        <f>D11+E11</f>
+        <v>2362.4593048095703</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update notes: 10-09-2026 20:36
</commit_message>
<xml_diff>
--- a/Time Series/moving_average.xlsx
+++ b/Time Series/moving_average.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MSQF\Semester III\Time Series\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8BECB8D-BC4B-48E4-A6EE-7AA0953E898E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71FFB607-E55E-4977-B6A4-2EB975FC0C46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Moving Average" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="04-09" sheetId="4" r:id="rId4"/>
     <sheet name="07-09" sheetId="5" r:id="rId5"/>
     <sheet name="09-09" sheetId="7" r:id="rId6"/>
+    <sheet name="10-09" sheetId="8" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="70">
   <si>
     <t>Year</t>
   </si>
@@ -204,12 +205,58 @@
   </si>
   <si>
     <t>Smoothed (alpha = 0.5)</t>
+  </si>
+  <si>
+    <t>AVERAGE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total average = </t>
+  </si>
+  <si>
+    <t>SEASONAL INDEX</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>DESEASONALIZED DATA</t>
+  </si>
+  <si>
+    <t>At</t>
+  </si>
+  <si>
+    <t>Ft (alpha = 0.5)</t>
+  </si>
+  <si>
+    <t>Ft (alpha = 1)</t>
+  </si>
+  <si>
+    <t>Ft (alpha = 0)</t>
+  </si>
+  <si>
+    <t>EXPONENTIAL SMOOTHING METHOD (SINGLE)</t>
+  </si>
+  <si>
+    <t>EXPONENTIAL SMOOTHING METHOD (DOUBLE)</t>
+  </si>
+  <si>
+    <t>Lt</t>
+  </si>
+  <si>
+    <t>Tt</t>
+  </si>
+  <si>
+    <t>Ft</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+  </numFmts>
   <fonts count="5">
     <font>
       <sz val="11"/>
@@ -331,7 +378,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -405,6 +452,17 @@
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1619,6 +1677,99 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>133624</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>123874</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A1521824-404E-507A-0D6F-AB9B84C48AE2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5486400" y="3962400"/>
+          <a:ext cx="1962424" cy="352474"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>391151</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>124141</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D155643E-70C5-0ADE-27DE-17B353AE6514}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4591050" y="5133975"/>
+          <a:ext cx="4486901" cy="2267266"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
   <a:themeElements>
@@ -4118,7 +4269,7 @@
         <v>12</v>
       </c>
       <c r="F3" s="27">
-        <f>D2+E2</f>
+        <f t="shared" ref="F3:F12" si="0">D2+E2</f>
         <v>1451</v>
       </c>
     </row>
@@ -4133,15 +4284,15 @@
         <v>1686</v>
       </c>
       <c r="D4" s="27">
-        <f t="shared" ref="D4:D11" si="0">0.5*C4+(1-0.5)*(D3+E3)</f>
+        <f t="shared" ref="D4:D11" si="1">0.5*C4+(1-0.5)*(D3+E3)</f>
         <v>1586.5</v>
       </c>
       <c r="E4" s="27">
-        <f t="shared" ref="E4:E11" si="1">0.5*(D4-D3)+(1-0.5)*E3</f>
+        <f t="shared" ref="E4:E11" si="2">0.5*(D4-D3)+(1-0.5)*E3</f>
         <v>61.75</v>
       </c>
       <c r="F4" s="27">
-        <f>D3+E3</f>
+        <f t="shared" si="0"/>
         <v>1487</v>
       </c>
     </row>
@@ -4156,15 +4307,15 @@
         <v>1764</v>
       </c>
       <c r="D5" s="27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1706.125</v>
       </c>
       <c r="E5" s="27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>90.6875</v>
       </c>
       <c r="F5" s="27">
-        <f>D4+E4</f>
+        <f t="shared" si="0"/>
         <v>1648.25</v>
       </c>
     </row>
@@ -4179,15 +4330,15 @@
         <v>1879</v>
       </c>
       <c r="D6" s="27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1837.90625</v>
       </c>
       <c r="E6" s="27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>111.234375</v>
       </c>
       <c r="F6" s="27">
-        <f>D5+E5</f>
+        <f t="shared" si="0"/>
         <v>1796.8125</v>
       </c>
     </row>
@@ -4202,15 +4353,15 @@
         <v>1948</v>
       </c>
       <c r="D7" s="27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1948.5703125</v>
       </c>
       <c r="E7" s="27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>110.94921875</v>
       </c>
       <c r="F7" s="27">
-        <f>D6+E6</f>
+        <f t="shared" si="0"/>
         <v>1949.140625</v>
       </c>
     </row>
@@ -4225,15 +4376,15 @@
         <v>2013</v>
       </c>
       <c r="D8" s="27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2036.259765625</v>
       </c>
       <c r="E8" s="27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>99.3193359375</v>
       </c>
       <c r="F8" s="27">
-        <f>D7+E7</f>
+        <f t="shared" si="0"/>
         <v>2059.51953125</v>
       </c>
     </row>
@@ -4248,15 +4399,15 @@
         <v>2090</v>
       </c>
       <c r="D9" s="27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2112.78955078125</v>
       </c>
       <c r="E9" s="27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>87.924560546875</v>
       </c>
       <c r="F9" s="27">
-        <f>D8+E8</f>
+        <f t="shared" si="0"/>
         <v>2135.5791015625</v>
       </c>
     </row>
@@ -4271,15 +4422,15 @@
         <v>2173</v>
       </c>
       <c r="D10" s="27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2186.8570556640625</v>
       </c>
       <c r="E10" s="27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>80.99603271484375</v>
       </c>
       <c r="F10" s="27">
-        <f>D9+E9</f>
+        <f t="shared" si="0"/>
         <v>2200.714111328125</v>
       </c>
     </row>
@@ -4294,15 +4445,15 @@
         <v>2286</v>
       </c>
       <c r="D11" s="27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2276.9265441894531</v>
       </c>
       <c r="E11" s="27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>85.532760620117188</v>
       </c>
       <c r="F11" s="27">
-        <f>D10+E10</f>
+        <f t="shared" si="0"/>
         <v>2267.8530883789063</v>
       </c>
     </row>
@@ -4314,11 +4465,524 @@
         <v>2020</v>
       </c>
       <c r="F12" s="27">
-        <f>D11+E11</f>
+        <f t="shared" si="0"/>
         <v>2362.4593048095703</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26533D8C-583C-4382-829E-773D66918166}">
+  <dimension ref="A1:I34"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="14.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="11.75" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15">
+      <c r="A1" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="B2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3">
+        <v>2011</v>
+      </c>
+      <c r="B3" s="28">
+        <v>3.7</v>
+      </c>
+      <c r="C3" s="28">
+        <v>4.7</v>
+      </c>
+      <c r="D3" s="28">
+        <v>3.3</v>
+      </c>
+      <c r="E3" s="28">
+        <v>3.5</v>
+      </c>
+      <c r="G3" s="31" t="s">
+        <v>43</v>
+      </c>
+      <c r="H3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3">
+        <f>B7/$B$9</f>
+        <v>0.97674418604651181</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4">
+        <v>2012</v>
+      </c>
+      <c r="B4" s="28">
+        <v>3.7</v>
+      </c>
+      <c r="C4" s="28">
+        <v>3.9</v>
+      </c>
+      <c r="D4" s="28">
+        <v>3.6</v>
+      </c>
+      <c r="E4" s="28">
+        <v>3.6</v>
+      </c>
+      <c r="G4" s="31"/>
+      <c r="H4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4">
+        <f>C7/$B$9</f>
+        <v>1.1362126245847179</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5">
+        <v>2013</v>
+      </c>
+      <c r="B5" s="28">
+        <v>4</v>
+      </c>
+      <c r="C5" s="28">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="D5" s="28">
+        <v>3.3</v>
+      </c>
+      <c r="E5" s="28">
+        <v>3.1</v>
+      </c>
+      <c r="G5" s="31"/>
+      <c r="H5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5">
+        <f>D7/$B$9</f>
+        <v>0.94352159468438557</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6">
+        <v>2014</v>
+      </c>
+      <c r="B6" s="28">
+        <v>3.3</v>
+      </c>
+      <c r="C6" s="28">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="D6" s="28">
+        <v>4</v>
+      </c>
+      <c r="E6" s="28">
+        <v>4</v>
+      </c>
+      <c r="G6" s="31"/>
+      <c r="H6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6">
+        <f>E7/$B$9</f>
+        <v>0.94352159468438557</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="28">
+        <f>AVERAGE(B3:B6)</f>
+        <v>3.6749999999999998</v>
+      </c>
+      <c r="C7" s="28">
+        <f t="shared" ref="C7:E7" si="0">AVERAGE(C3:C6)</f>
+        <v>4.2750000000000004</v>
+      </c>
+      <c r="D7" s="28">
+        <f t="shared" si="0"/>
+        <v>3.55</v>
+      </c>
+      <c r="E7" s="28">
+        <f t="shared" si="0"/>
+        <v>3.55</v>
+      </c>
+      <c r="H7" t="s">
+        <v>59</v>
+      </c>
+      <c r="I7">
+        <f>SUM(I3:I6)</f>
+        <v>4.0000000000000009</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="28">
+        <f>AVERAGE(B3:E7)</f>
+        <v>3.7624999999999993</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="15">
+      <c r="A12" s="32" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" s="32"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="32"/>
+      <c r="I12" s="32"/>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="B14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15">
+        <v>2011</v>
+      </c>
+      <c r="B15" s="30">
+        <f>B3/$I$3</f>
+        <v>3.7880952380952375</v>
+      </c>
+      <c r="C15" s="30">
+        <f>C3/$I$4</f>
+        <v>4.1365497076023381</v>
+      </c>
+      <c r="D15" s="30">
+        <f>D3/$I$5</f>
+        <v>3.4975352112676048</v>
+      </c>
+      <c r="E15" s="30">
+        <f>E3/$I$6</f>
+        <v>3.7095070422535206</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16">
+        <v>2012</v>
+      </c>
+      <c r="B16" s="30">
+        <f t="shared" ref="B16:B18" si="1">B4/$I$3</f>
+        <v>3.7880952380952375</v>
+      </c>
+      <c r="C16" s="30">
+        <f t="shared" ref="C16:C18" si="2">C4/$I$4</f>
+        <v>3.432456140350876</v>
+      </c>
+      <c r="D16" s="30">
+        <f t="shared" ref="D16:D18" si="3">D4/$I$5</f>
+        <v>3.815492957746478</v>
+      </c>
+      <c r="E16" s="30">
+        <f t="shared" ref="E16:E18" si="4">E4/$I$6</f>
+        <v>3.815492957746478</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17">
+        <v>2013</v>
+      </c>
+      <c r="B17" s="30">
+        <f t="shared" si="1"/>
+        <v>4.0952380952380949</v>
+      </c>
+      <c r="C17" s="30">
+        <f t="shared" si="2"/>
+        <v>3.6084795321637415</v>
+      </c>
+      <c r="D17" s="30">
+        <f t="shared" si="3"/>
+        <v>3.4975352112676048</v>
+      </c>
+      <c r="E17" s="30">
+        <f t="shared" si="4"/>
+        <v>3.2855633802816895</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18">
+        <v>2014</v>
+      </c>
+      <c r="B18" s="30">
+        <f t="shared" si="1"/>
+        <v>3.3785714285714277</v>
+      </c>
+      <c r="C18" s="30">
+        <f t="shared" si="2"/>
+        <v>3.8725146198830402</v>
+      </c>
+      <c r="D18" s="30">
+        <f t="shared" si="3"/>
+        <v>4.2394366197183091</v>
+      </c>
+      <c r="E18" s="30">
+        <f t="shared" si="4"/>
+        <v>4.2394366197183091</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="15">
+      <c r="A21" s="32" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" s="32"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="C22" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D22" s="29" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="29">
+        <v>1.2</v>
+      </c>
+      <c r="B23" s="29">
+        <f>A23</f>
+        <v>1.2</v>
+      </c>
+      <c r="C23" s="29">
+        <f>A23</f>
+        <v>1.2</v>
+      </c>
+      <c r="D23" s="26">
+        <f>A23</f>
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="29">
+        <v>0.9</v>
+      </c>
+      <c r="B24" s="29">
+        <f>0.5*A23+(1-0.5)*B23</f>
+        <v>1.2</v>
+      </c>
+      <c r="C24" s="29">
+        <f>1*A23+(1-1)*B23</f>
+        <v>1.2</v>
+      </c>
+      <c r="D24" s="26">
+        <f>0*A23+(1-0)*B23</f>
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="29">
+        <v>0.7</v>
+      </c>
+      <c r="B25" s="29">
+        <f t="shared" ref="B25:B26" si="5">0.5*A24+(1-0.5)*B24</f>
+        <v>1.05</v>
+      </c>
+      <c r="C25" s="29">
+        <f t="shared" ref="C25:C26" si="6">1*A24+(1-1)*B24</f>
+        <v>0.9</v>
+      </c>
+      <c r="D25" s="26">
+        <f t="shared" ref="D25:D26" si="7">0*A24+(1-0)*B24</f>
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="29">
+        <v>1.3</v>
+      </c>
+      <c r="B26" s="29">
+        <f t="shared" si="5"/>
+        <v>0.875</v>
+      </c>
+      <c r="C26" s="29">
+        <f t="shared" si="6"/>
+        <v>0.7</v>
+      </c>
+      <c r="D26" s="26">
+        <f t="shared" si="7"/>
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="15">
+      <c r="A28" s="32" t="s">
+        <v>66</v>
+      </c>
+      <c r="B28" s="32"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="32"/>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="C29" s="29" t="s">
+        <v>68</v>
+      </c>
+      <c r="D29" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="E29" s="29"/>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" s="29">
+        <v>64</v>
+      </c>
+      <c r="B30" s="29">
+        <f>A30</f>
+        <v>64</v>
+      </c>
+      <c r="C30" s="29">
+        <f>A31-A30</f>
+        <v>18</v>
+      </c>
+      <c r="D30" s="29">
+        <v>0</v>
+      </c>
+      <c r="E30" s="29"/>
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31" s="29">
+        <v>82</v>
+      </c>
+      <c r="B31" s="29">
+        <f>0.5*A31+(1-0.5)*(B30+C30)</f>
+        <v>82</v>
+      </c>
+      <c r="C31" s="29">
+        <f>0.5*(B31-B30)+(1-0.5)*C30</f>
+        <v>18</v>
+      </c>
+      <c r="D31" s="29">
+        <f>B31+C31</f>
+        <v>100</v>
+      </c>
+      <c r="E31" s="29"/>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" s="29">
+        <v>92</v>
+      </c>
+      <c r="B32" s="29">
+        <f t="shared" ref="B32:B34" si="8">0.5*A32+(1-0.5)*(B31+C31)</f>
+        <v>96</v>
+      </c>
+      <c r="C32" s="29">
+        <f t="shared" ref="C32:C34" si="9">0.5*(B32-B31)+(1-0.5)*C31</f>
+        <v>16</v>
+      </c>
+      <c r="D32" s="29">
+        <f t="shared" ref="D32:D34" si="10">B32+C32</f>
+        <v>112</v>
+      </c>
+      <c r="E32" s="29"/>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" s="29">
+        <v>95</v>
+      </c>
+      <c r="B33" s="29">
+        <f t="shared" si="8"/>
+        <v>103.5</v>
+      </c>
+      <c r="C33" s="29">
+        <f t="shared" si="9"/>
+        <v>11.75</v>
+      </c>
+      <c r="D33" s="29">
+        <f t="shared" si="10"/>
+        <v>115.25</v>
+      </c>
+      <c r="E33" s="29"/>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" s="29">
+        <v>106</v>
+      </c>
+      <c r="B34" s="29">
+        <f t="shared" si="8"/>
+        <v>110.625</v>
+      </c>
+      <c r="C34" s="29">
+        <f t="shared" si="9"/>
+        <v>9.4375</v>
+      </c>
+      <c r="D34" s="29">
+        <f t="shared" si="10"/>
+        <v>120.0625</v>
+      </c>
+      <c r="E34" s="29"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="G3:G6"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A28:I28"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>